<commit_message>
IA con Groq para extracción de facturas
</commit_message>
<xml_diff>
--- a/backend/resultados.xlsx
+++ b/backend/resultados.xlsx
@@ -505,37 +505,37 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TechSoluciones S.L.</t>
+          <t>IONOS Cloud S.L.U.</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>B98765432</t>
+          <t>B-85049435</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2024-0142</t>
+          <t>202785775209</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>28/02/2024</t>
+          <t>06/03/26</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2350.00 EUR</t>
+          <t>51.00 EUR</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>493.50 EUR</t>
+          <t>10.71 EUR</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2843.50 EUR</t>
+          <t>61.71 EUR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mejora extracción emisor/cliente y toggle razón social
</commit_message>
<xml_diff>
--- a/backend/resultados.xlsx
+++ b/backend/resultados.xlsx
@@ -505,37 +505,37 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IONOS Cloud S.L.U.</t>
+          <t>ALPESA</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>B-85049435</t>
+          <t>B18756734</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>202785775209</t>
+          <t>FP26-0026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>06/03/26</t>
+          <t>09/01/2026</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>51.00 EUR</t>
+          <t>150.27 EUR</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>10.71 EUR</t>
+          <t>31.56 EUR</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>61.71 EUR</t>
+          <t>181.83 EUR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Añadir contacto, testimonios y contador en landing
</commit_message>
<xml_diff>
--- a/backend/resultados.xlsx
+++ b/backend/resultados.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +51,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D6EAE4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,12 +85,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -453,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -505,35 +513,257 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>IONOS Cloud S.L.U.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>B-85049435</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>202785775209</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>06/03/26</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>51.00 EUR</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>10.71 EUR</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>61.71 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>SOLUCIONES DIGITALES ORBEX S.L.</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>B-84902177</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>F-2024/NOV/0087</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>14/11/2024</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>4815.10 EUR</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>1011.17 EUR</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>5826.27 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>FacturaAI S.L.</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>B87654321</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>FAI/2026/03/0042</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>5.462.50</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1.147.13</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>5.790.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Gestoría Ejemplo S.L.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>B12345678</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2026-001</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>08/03/2026</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>25.00 EUR</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>5.25 EUR</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>30.25 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TechSoluciones S.L.</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>B98765432</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>F-2024-0142</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>28/02/2024</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2350.00 EUR</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>493.50 EUR</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2843.50 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Closemarketing, SL</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>B19618909</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>H2026-002</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>28/02/2026</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>129.00 EUR</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>27.09 EUR</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>156.09 EUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>ALPESA</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>B18756734</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>FP26-0026</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>09/01/2026</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>150.27 EUR</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>31.56 EUR</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>181.83 EUR</t>
         </is>

</xml_diff>